<commit_message>
Add React deployment configuration and Selenium E2E testing framework with GitHub Actions
</commit_message>
<xml_diff>
--- a/EcoTrade_Test_Report.xlsx
+++ b/EcoTrade_Test_Report.xlsx
@@ -517,7 +517,7 @@
     <row r="3">
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Executed At: 2026-06-16 14:03:43 | Environment: Android Emulator &amp; Chrome Sandbox</t>
+          <t>Executed At: 2026-06-16 22:36:32 | Environment: Android Emulator &amp; Chrome Sandbox</t>
         </is>
       </c>
     </row>
@@ -578,7 +578,7 @@
       </c>
       <c r="C10" s="5" t="inlineStr">
         <is>
-          <t>6.21 seconds</t>
+          <t>5.78 seconds</t>
         </is>
       </c>
     </row>

</xml_diff>